<commit_message>
chore: sync MLA fee export updates
</commit_message>
<xml_diff>
--- a/outputs/ema-fee-detail-export/JLR- EMA 费用规则.xlsx
+++ b/outputs/ema-fee-detail-export/JLR- EMA 费用规则.xlsx
@@ -4561,7 +4561,7 @@
       </c>
       <c r="AB32" s="5" t="inlineStr">
         <is>
-          <t>Optical Test: baseline 汇总，51 点位样品按组各取 1 台，其余按 19 点位计费；Optical Test: 1 台按 51 点位，其余按 19 点位计费；Optical Test: 全部按 19 点位计费</t>
+          <t xml:space="preserve">Optical Test 特殊计算：51 点位 134/个，19 点位 50/个；普通组 1 台按 51 点位、其余按 19 点位，Group D-8 全部按 19 点位。</t>
         </is>
       </c>
       <c r="AC32" s="5" t="n">
@@ -4585,7 +4585,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15.2" outlineLevelRow="2"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4692,6 +4692,38 @@
         </is>
       </c>
     </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">V.2</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-17</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">费用规则修正</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">调整 Optical Test 特殊计费单价：19 点位由 210/个改为 50/个，51 点位由 460/个改为 134/个；AB列规则备注同步写明新单价和计算口径。</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">费用规则去重表!AB:AB；/environment-outline Optical Test 费用计算</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">对应系统本地草稿模板版本 ENVIRONMENT_PLAN_TEMPLATE_VERSION = 37。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>